<commit_message>
Include new model training datasets and outputs
</commit_message>
<xml_diff>
--- a/football_output_v2/readable/football_performance_report.xlsx
+++ b/football_output_v2/readable/football_performance_report.xlsx
@@ -8,7 +8,6 @@
     <sheet name="Calibration" sheetId="4" ns1:id="R6fe18dcc89cb4419"/>
     <sheet name="Selections" sheetId="5" ns1:id="R320e3c7a9bc644fa"/>
     <sheet name="Predictions" sheetId="6" ns1:id="Rcc8cb310aa834b56"/>
-    <sheet name="Pipeline Health" sheetId="7" ns1:id="rIdPipelineHealth"/>
   </sheets>
   <calcPr fullCalcOnLoad="1" calcMode="auto"/>
 </workbook>
@@ -12490,805 +12489,4 @@
     <tablePart ns1:id="Rab36e2e62cba44b5"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="52" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Pipeline health and forward evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Review UTC: 2026-10-13T11:48:17.228667+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Source freshness, model results and execution checks are separate evidence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>League</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Training end</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Matches</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Days since result</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Source status</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Bundesliga</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>963</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>EPL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>1200</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LaLiga</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>1218</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Ligue1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>972</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SerieA</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>1200</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>UCL</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>521</v>
-      </c>
-      <c r="D12">
-        <v>33</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>CURRENT_WITHIN_PROVIDER_SCHEDULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Latest stored shortlist audit</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>selected_quotes</t>
-        </is>
-      </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>exchange_quotes</t>
-        </is>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>missing_quote_age</t>
-        </is>
-      </c>
-      <c r="B17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>quote_age_over_24h</t>
-        </is>
-      </c>
-      <c r="B18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>costs_recorded</t>
-        </is>
-      </c>
-      <c r="B19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>bookmakers</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>{"Coolbet": 3, "Matchbook": 1, "1xBet": 1}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>account_availability</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>NOT_VERIFIED_WITH_BOOKMAKER_ACCOUNTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Snapshot</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Captured UTC</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Goal blend</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Market led</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2fd31d337223</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-10-11T06:30:30Z</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>bdc690a8c706</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026-10-11T06:38:09Z</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>b9c15c09504a</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-10-11T06:44:04Z</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>648ca5973f8d</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-10-11T08:21:00Z</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>660b75e4a311</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2026-10-11T08:25:02Z</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>a2cdead106b5</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026-10-11T10:46:00Z</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>5fb257972ff2</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2026-10-11T11:06:08Z</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>f1a72cc22d71</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>2026-10-11T11:32:53Z</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>4f7af2f470a0</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>2026-10-12T16:34:11Z</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>5496e9ba03ae</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2026-10-12T21:11:56Z</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>f6306ebd6d74</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2026-10-13T07:01:01Z</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>fbfe5af89d06</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>2026-10-13T07:52:43Z</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>87b1676077a4</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>2026-10-13T09:01:13Z</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>0dba961b0bbe</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>2026-10-13T09:27:14Z</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>LEGACY_NOT_RECORDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>962a7a22cb5b</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>2026-10-13T11:07:31Z</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>CAPTURED</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>CAPTURED</t>
-        </is>
-      </c>
-    </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Daily observations</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Graded</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Win rate</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Net simulated ROI</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Brier</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="B41">
-        <v>7</v>
-      </c>
-      <c r="C41">
-        <v>0.571429</v>
-      </c>
-      <c r="D41">
-        <v>-0.215714</v>
-      </c>
-      <c r="E41">
-        <v>0.309299</v>
-      </c>
-    </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Review dependency versions</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>3.12.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>numpy</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2.5.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>pandas</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>3.0.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>scipy</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>1.18.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>requests</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>2.34.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>python-dotenv</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>1.2.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>coverage</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>NOT_INSTALLED</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>PyYAML</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>NOT_INSTALLED</t>
-        </is>
-      </c>
-    </row>
-    <row r="52"/>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Improvement is not established by fresher data or software changes. Compare paired forecasts and settled results.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Account access and executable stake sizes are not verified. Exchange targets require a commission/liquidity adapter.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Include model training data and outputs
</commit_message>
<xml_diff>
--- a/football_output_v2/readable/football_performance_report.xlsx
+++ b/football_output_v2/readable/football_performance_report.xlsx
@@ -5424,113 +5424,113 @@
     <row r="38" ht="44" customHeight="1">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>Selected quotes</t>
-        </is>
-      </c>
-      <c r="B38" s="19">
-        <v>6</v>
+          <t>Account availability</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>Not verified with bookmaker accounts</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>Exchange quotes</t>
+          <t>Bookmakers: 1xBet</t>
         </is>
       </c>
       <c r="B39" s="19">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>Missing quote age</t>
+          <t>Bookmakers: Pinnacle</t>
         </is>
       </c>
       <c r="B40" s="19">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>Quote age over 24h</t>
+          <t>Costs recorded</t>
         </is>
       </c>
       <c r="B41" s="19">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>Costs recorded</t>
+          <t>Exchange quotes</t>
         </is>
       </c>
       <c r="B42" s="19">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>Bookmakers: 1xBet</t>
+          <t>Missing quote age</t>
         </is>
       </c>
       <c r="B43" s="19">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>Bookmakers: Pinnacle</t>
+          <t>Past kickoff count</t>
         </is>
       </c>
       <c r="B44" s="19">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>Account availability</t>
-        </is>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
-        <is>
-          <t>Not verified with bookmaker accounts</t>
-        </is>
+          <t>Quote age over 24h</t>
+        </is>
+      </c>
+      <c r="B45" s="19">
+        <v>0</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>Past kickoff count</t>
+          <t>Selected quotes</t>
         </is>
       </c>
       <c r="B46" s="19">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>Upcoming kickoff count</t>
+          <t>Unknown kickoff count</t>
         </is>
       </c>
       <c r="B47" s="19">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>Unknown kickoff count</t>
+          <t>Upcoming kickoff count</t>
         </is>
       </c>
       <c r="B48" s="19">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51">
@@ -6404,108 +6404,108 @@
     <row r="108" ht="44" customHeight="1">
       <c r="A108" s="18" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>PyYAML</t>
         </is>
       </c>
       <c r="B108" s="18" t="inlineStr">
         <is>
-          <t>3.12.15</t>
+          <t>6.0.3</t>
         </is>
       </c>
     </row>
     <row r="109" ht="44" customHeight="1">
       <c r="A109" s="18" t="inlineStr">
         <is>
-          <t>numpy</t>
+          <t>coverage</t>
         </is>
       </c>
       <c r="B109" s="18" t="inlineStr">
         <is>
-          <t>2.5.4</t>
+          <t>7.17.0</t>
         </is>
       </c>
     </row>
     <row r="110" ht="44" customHeight="1">
       <c r="A110" s="18" t="inlineStr">
         <is>
-          <t>pandas</t>
+          <t>numpy</t>
         </is>
       </c>
       <c r="B110" s="18" t="inlineStr">
         <is>
-          <t>3.1.0</t>
+          <t>2.5.4</t>
         </is>
       </c>
     </row>
     <row r="111" ht="44" customHeight="1">
       <c r="A111" s="18" t="inlineStr">
         <is>
-          <t>scipy</t>
+          <t>pandas</t>
         </is>
       </c>
       <c r="B111" s="18" t="inlineStr">
         <is>
-          <t>1.18.1</t>
+          <t>3.1.0</t>
         </is>
       </c>
     </row>
     <row r="112" ht="44" customHeight="1">
       <c r="A112" s="18" t="inlineStr">
         <is>
-          <t>requests</t>
+          <t>python</t>
         </is>
       </c>
       <c r="B112" s="18" t="inlineStr">
         <is>
-          <t>2.34.2</t>
+          <t>3.12.15</t>
         </is>
       </c>
     </row>
     <row r="113" ht="44" customHeight="1">
       <c r="A113" s="18" t="inlineStr">
         <is>
-          <t>rapidfuzz</t>
+          <t>python-dotenv</t>
         </is>
       </c>
       <c r="B113" s="18" t="inlineStr">
         <is>
-          <t>3.14.6</t>
+          <t>1.2.4</t>
         </is>
       </c>
     </row>
     <row r="114" ht="44" customHeight="1">
       <c r="A114" s="18" t="inlineStr">
         <is>
-          <t>python-dotenv</t>
+          <t>rapidfuzz</t>
         </is>
       </c>
       <c r="B114" s="18" t="inlineStr">
         <is>
-          <t>1.2.4</t>
+          <t>3.14.6</t>
         </is>
       </c>
     </row>
     <row r="115" ht="44" customHeight="1">
       <c r="A115" s="18" t="inlineStr">
         <is>
-          <t>coverage</t>
+          <t>requests</t>
         </is>
       </c>
       <c r="B115" s="18" t="inlineStr">
         <is>
-          <t>7.17.0</t>
+          <t>2.34.2</t>
         </is>
       </c>
     </row>
     <row r="116" ht="44" customHeight="1">
       <c r="A116" s="18" t="inlineStr">
         <is>
-          <t>PyYAML</t>
+          <t>scipy</t>
         </is>
       </c>
       <c r="B116" s="18" t="inlineStr">
         <is>
-          <t>6.0.3</t>
+          <t>1.18.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Initial commit excluding heavy models
</commit_message>
<xml_diff>
--- a/football_output_v2/readable/football_performance_report.xlsx
+++ b/football_output_v2/readable/football_performance_report.xlsx
@@ -6065,37 +6065,39 @@
     <row r="46" ht="44" customHeight="1">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>Selected quotes</t>
-        </is>
-      </c>
-      <c r="B46" s="19">
-        <v>1</v>
+          <t>Account availability</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>Not verified with bookmaker accounts</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>Exchange quotes</t>
+          <t>Bookmakers: Pinnacle</t>
         </is>
       </c>
       <c r="B47" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>Missing quote age</t>
+          <t>Costs recorded</t>
         </is>
       </c>
       <c r="B48" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>Quote age over 24h</t>
+          <t>Exchange quotes</t>
         </is>
       </c>
       <c r="B49" s="19">
@@ -6105,63 +6107,61 @@
     <row r="50" ht="44" customHeight="1">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>Costs recorded</t>
+          <t>Missing quote age</t>
         </is>
       </c>
       <c r="B50" s="19">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>Bookmakers: Pinnacle</t>
+          <t>Past kickoff count</t>
         </is>
       </c>
       <c r="B51" s="19">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>Account availability</t>
-        </is>
-      </c>
-      <c r="B52" s="18" t="inlineStr">
-        <is>
-          <t>Not verified with bookmaker accounts</t>
-        </is>
+          <t>Quote age over 24h</t>
+        </is>
+      </c>
+      <c r="B52" s="19">
+        <v>0</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>Past kickoff count</t>
+          <t>Selected quotes</t>
         </is>
       </c>
       <c r="B53" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>Upcoming kickoff count</t>
+          <t>Unknown kickoff count</t>
         </is>
       </c>
       <c r="B54" s="19">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1">
       <c r="A55" s="18" t="inlineStr">
         <is>
-          <t>Unknown kickoff count</t>
+          <t>Upcoming kickoff count</t>
         </is>
       </c>
       <c r="B55" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -7130,108 +7130,108 @@
     <row r="120" ht="44" customHeight="1">
       <c r="A120" s="18" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>PyYAML</t>
         </is>
       </c>
       <c r="B120" s="18" t="inlineStr">
         <is>
-          <t>3.12.15</t>
+          <t>NOT_INSTALLED</t>
         </is>
       </c>
     </row>
     <row r="121" ht="44" customHeight="1">
       <c r="A121" s="18" t="inlineStr">
         <is>
-          <t>numpy</t>
+          <t>coverage</t>
         </is>
       </c>
       <c r="B121" s="18" t="inlineStr">
         <is>
-          <t>2.5.4</t>
+          <t>NOT_INSTALLED</t>
         </is>
       </c>
     </row>
     <row r="122" ht="44" customHeight="1">
       <c r="A122" s="18" t="inlineStr">
         <is>
-          <t>pandas</t>
+          <t>numpy</t>
         </is>
       </c>
       <c r="B122" s="18" t="inlineStr">
         <is>
-          <t>3.1.0</t>
+          <t>2.5.4</t>
         </is>
       </c>
     </row>
     <row r="123" ht="44" customHeight="1">
       <c r="A123" s="18" t="inlineStr">
         <is>
-          <t>scipy</t>
+          <t>pandas</t>
         </is>
       </c>
       <c r="B123" s="18" t="inlineStr">
         <is>
-          <t>1.18.1</t>
+          <t>3.1.0</t>
         </is>
       </c>
     </row>
     <row r="124" ht="44" customHeight="1">
       <c r="A124" s="18" t="inlineStr">
         <is>
-          <t>requests</t>
+          <t>python</t>
         </is>
       </c>
       <c r="B124" s="18" t="inlineStr">
         <is>
-          <t>2.34.2</t>
+          <t>3.12.15</t>
         </is>
       </c>
     </row>
     <row r="125" ht="44" customHeight="1">
       <c r="A125" s="18" t="inlineStr">
         <is>
-          <t>rapidfuzz</t>
+          <t>python-dotenv</t>
         </is>
       </c>
       <c r="B125" s="18" t="inlineStr">
         <is>
-          <t>3.14.6</t>
+          <t>1.2.4</t>
         </is>
       </c>
     </row>
     <row r="126" ht="44" customHeight="1">
       <c r="A126" s="18" t="inlineStr">
         <is>
-          <t>python-dotenv</t>
+          <t>rapidfuzz</t>
         </is>
       </c>
       <c r="B126" s="18" t="inlineStr">
         <is>
-          <t>1.2.4</t>
+          <t>3.14.6</t>
         </is>
       </c>
     </row>
     <row r="127" ht="44" customHeight="1">
       <c r="A127" s="18" t="inlineStr">
         <is>
-          <t>coverage</t>
+          <t>requests</t>
         </is>
       </c>
       <c r="B127" s="18" t="inlineStr">
         <is>
-          <t>NOT_INSTALLED</t>
+          <t>2.34.2</t>
         </is>
       </c>
     </row>
     <row r="128" ht="44" customHeight="1">
       <c r="A128" s="18" t="inlineStr">
         <is>
-          <t>PyYAML</t>
+          <t>scipy</t>
         </is>
       </c>
       <c r="B128" s="18" t="inlineStr">
         <is>
-          <t>NOT_INSTALLED</t>
+          <t>1.18.1</t>
         </is>
       </c>
     </row>

</xml_diff>